<commit_message>
Persist allocation results in AllocationState and cleanup dashboard
Updated AllocationState to store the latest capacities and results, and ensured these are updated after allocation in the Controller. Cleaned up WarehouseDashboard component by removing commented mock data and minor formatting. Minor code improvements in DashboardController and App.tsx. Updated output Excel file with new allocation results.
</commit_message>
<xml_diff>
--- a/outputFile/AllocatedResult2025DENMARK.xlsx
+++ b/outputFile/AllocatedResult2025DENMARK.xlsx
@@ -12,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3" uniqueCount="3">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="45" uniqueCount="9">
   <si>
     <t>Warehouse</t>
   </si>
@@ -21,6 +21,24 @@
   </si>
   <si>
     <t>Amount Stored</t>
+  </si>
+  <si>
+    <t>NEFF</t>
+  </si>
+  <si>
+    <t>FREEZE</t>
+  </si>
+  <si>
+    <t>PS PAC II</t>
+  </si>
+  <si>
+    <t>AMBIENT</t>
+  </si>
+  <si>
+    <t>COLD</t>
+  </si>
+  <si>
+    <t>PS PAC I</t>
   </si>
 </sst>
 </file>
@@ -65,7 +83,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:C1"/>
+  <dimension ref="A1:C22"/>
   <sheetFormatPr defaultRowHeight="15.0"/>
   <sheetData>
     <row r="1">
@@ -79,6 +97,237 @@
         <v>2</v>
       </c>
     </row>
+    <row r="2">
+      <c r="A2" t="s" s="0">
+        <v>3</v>
+      </c>
+      <c r="B2" t="s" s="0">
+        <v>4</v>
+      </c>
+      <c r="C2" t="n" s="0">
+        <v>1414.0</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="s" s="0">
+        <v>5</v>
+      </c>
+      <c r="B3" t="s" s="0">
+        <v>6</v>
+      </c>
+      <c r="C3" t="n" s="0">
+        <v>200.0</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="s" s="0">
+        <v>5</v>
+      </c>
+      <c r="B4" t="s" s="0">
+        <v>6</v>
+      </c>
+      <c r="C4" t="n" s="0">
+        <v>220.0</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="s" s="0">
+        <v>3</v>
+      </c>
+      <c r="B5" t="s" s="0">
+        <v>7</v>
+      </c>
+      <c r="C5" t="n" s="0">
+        <v>2393.0</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="s" s="0">
+        <v>3</v>
+      </c>
+      <c r="B6" t="s" s="0">
+        <v>7</v>
+      </c>
+      <c r="C6" t="n" s="0">
+        <v>9074.0</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="s" s="0">
+        <v>3</v>
+      </c>
+      <c r="B7" t="s" s="0">
+        <v>7</v>
+      </c>
+      <c r="C7" t="n" s="0">
+        <v>450.0</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="s" s="0">
+        <v>8</v>
+      </c>
+      <c r="B8" t="s" s="0">
+        <v>6</v>
+      </c>
+      <c r="C8" t="n" s="0">
+        <v>12575.0</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="s" s="0">
+        <v>5</v>
+      </c>
+      <c r="B9" t="s" s="0">
+        <v>6</v>
+      </c>
+      <c r="C9" t="n" s="0">
+        <v>15953.0</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="s" s="0">
+        <v>3</v>
+      </c>
+      <c r="B10" t="s" s="0">
+        <v>6</v>
+      </c>
+      <c r="C10" t="n" s="0">
+        <v>9295.0</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="s" s="0">
+        <v>5</v>
+      </c>
+      <c r="B11" t="s" s="0">
+        <v>6</v>
+      </c>
+      <c r="C11" t="n" s="0">
+        <v>3800.0</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="s" s="0">
+        <v>8</v>
+      </c>
+      <c r="B12" t="s" s="0">
+        <v>6</v>
+      </c>
+      <c r="C12" t="n" s="0">
+        <v>6886.0</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="s" s="0">
+        <v>8</v>
+      </c>
+      <c r="B13" t="s" s="0">
+        <v>6</v>
+      </c>
+      <c r="C13" t="n" s="0">
+        <v>886.0</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="s" s="0">
+        <v>8</v>
+      </c>
+      <c r="B14" t="s" s="0">
+        <v>6</v>
+      </c>
+      <c r="C14" t="n" s="0">
+        <v>300.0</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="s" s="0">
+        <v>3</v>
+      </c>
+      <c r="B15" t="s" s="0">
+        <v>6</v>
+      </c>
+      <c r="C15" t="n" s="0">
+        <v>2500.0</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="s" s="0">
+        <v>5</v>
+      </c>
+      <c r="B16" t="s" s="0">
+        <v>6</v>
+      </c>
+      <c r="C16" t="n" s="0">
+        <v>600.0</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="s" s="0">
+        <v>5</v>
+      </c>
+      <c r="B17" t="s" s="0">
+        <v>6</v>
+      </c>
+      <c r="C17" t="n" s="0">
+        <v>15000.0</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="s" s="0">
+        <v>3</v>
+      </c>
+      <c r="B18" t="s" s="0">
+        <v>7</v>
+      </c>
+      <c r="C18" t="n" s="0">
+        <v>200.0</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="s" s="0">
+        <v>3</v>
+      </c>
+      <c r="B19" t="s" s="0">
+        <v>4</v>
+      </c>
+      <c r="C19" t="n" s="0">
+        <v>1300.0</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="s" s="0">
+        <v>5</v>
+      </c>
+      <c r="B20" t="s" s="0">
+        <v>6</v>
+      </c>
+      <c r="C20" t="n" s="0">
+        <v>100.0</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="s" s="0">
+        <v>3</v>
+      </c>
+      <c r="B21" t="s" s="0">
+        <v>7</v>
+      </c>
+      <c r="C21" t="n" s="0">
+        <v>430.0</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="s" s="0">
+        <v>3</v>
+      </c>
+      <c r="B22" t="s" s="0">
+        <v>7</v>
+      </c>
+      <c r="C22" t="n" s="0">
+        <v>54.0</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins bottom="0.75" footer="0.3" header="0.3" left="0.7" right="0.7" top="0.75"/>
 </worksheet>

</xml_diff>